<commit_message>
updated compass_mot_pinning to account for Ark Mag
</commit_message>
<xml_diff>
--- a/doc/params/xplorer-params-DEV.xlsx
+++ b/doc/params/xplorer-params-DEV.xlsx
@@ -15354,7 +15354,7 @@
         </is>
       </c>
       <c r="C274" t="n">
-        <v>96515</v>
+        <v>96259</v>
       </c>
       <c r="D274" t="b">
         <v>0</v>
@@ -15404,7 +15404,7 @@
         </is>
       </c>
       <c r="C275" t="n">
-        <v>162051</v>
+        <v>96515</v>
       </c>
       <c r="D275" t="b">
         <v>0</v>
@@ -15454,7 +15454,7 @@
         </is>
       </c>
       <c r="C276" t="n">
-        <v>1313809</v>
+        <v>0</v>
       </c>
       <c r="D276" t="b">
         <v>0</v>
@@ -15483,7 +15483,7 @@
       <c r="P276" t="inlineStr"/>
       <c r="Q276" t="inlineStr">
         <is>
-          <t>defaults.parm: # TEMP-COMPASS-EXPERIMENT unlocked</t>
+          <t>defaults.parm: # TEMP-COMPASS-EXPERIMENT unlocked | Deliberately seeded 0 - see COMPASS_PRIO3_ID. Slot 3 is left floating.</t>
         </is>
       </c>
       <c r="R276" t="inlineStr">
@@ -16593,7 +16593,7 @@
       <c r="P298" t="inlineStr"/>
       <c r="Q298" t="inlineStr">
         <is>
-          <t>NOT SEEDED - compassmot compensation. Device-ID pinning table exists (ArduCopter/xplorer_compass_mot_pinning.h) but xplorer_compass_mot_boot_align() is CURRENTLY COMMENTED OUT in system.cpp (TEMP-COMPASS-EXPERIMENT) | should make false once we fix this on a lower level</t>
+          <t>NOT SEEDED in defaults.parm - value is written at boot by xplorer_compass_mot_boot_align() (system.cpp) from the device-ID-keyed table in ArduCopter/xplorer_compass_mot_pinning.h, which is the source of truth. Running CompassMot on a deployed unit will NOT persist across reboot; update the table and rebuild instead.</t>
         </is>
       </c>
       <c r="R298" t="inlineStr">
@@ -16654,7 +16654,7 @@
       <c r="P299" t="inlineStr"/>
       <c r="Q299" t="inlineStr">
         <is>
-          <t>NOT SEEDED - compassmot compensation. Device-ID pinning table exists (ArduCopter/xplorer_compass_mot_pinning.h) but xplorer_compass_mot_boot_align() is CURRENTLY COMMENTED OUT in system.cpp (TEMP-COMPASS-EXPERIMENT) | should make false once we fix this on a lower level</t>
+          <t>NOT SEEDED in defaults.parm - value is written at boot by xplorer_compass_mot_boot_align() (system.cpp) from the device-ID-keyed table in ArduCopter/xplorer_compass_mot_pinning.h, which is the source of truth. Running CompassMot on a deployed unit will NOT persist across reboot; update the table and rebuild instead.</t>
         </is>
       </c>
       <c r="R299" t="inlineStr">
@@ -16715,7 +16715,7 @@
       <c r="P300" t="inlineStr"/>
       <c r="Q300" t="inlineStr">
         <is>
-          <t>NOT SEEDED - compassmot compensation. Device-ID pinning table exists (ArduCopter/xplorer_compass_mot_pinning.h) but xplorer_compass_mot_boot_align() is CURRENTLY COMMENTED OUT in system.cpp (TEMP-COMPASS-EXPERIMENT) | should make false once we fix this on a lower level</t>
+          <t>NOT SEEDED in defaults.parm - value is written at boot by xplorer_compass_mot_boot_align() (system.cpp) from the device-ID-keyed table in ArduCopter/xplorer_compass_mot_pinning.h, which is the source of truth. Running CompassMot on a deployed unit will NOT persist across reboot; update the table and rebuild instead.</t>
         </is>
       </c>
       <c r="R300" t="inlineStr">
@@ -16776,7 +16776,7 @@
       <c r="P301" t="inlineStr"/>
       <c r="Q301" t="inlineStr">
         <is>
-          <t>NOT SEEDED - compassmot compensation. Device-ID pinning table exists (ArduCopter/xplorer_compass_mot_pinning.h) but xplorer_compass_mot_boot_align() is CURRENTLY COMMENTED OUT in system.cpp (TEMP-COMPASS-EXPERIMENT) | should make false once we fix this on a lower level</t>
+          <t>NOT SEEDED in defaults.parm - value is written at boot by xplorer_compass_mot_boot_align() (system.cpp) from the device-ID-keyed table in ArduCopter/xplorer_compass_mot_pinning.h, which is the source of truth. Running CompassMot on a deployed unit will NOT persist across reboot; update the table and rebuild instead.</t>
         </is>
       </c>
       <c r="R301" t="inlineStr">
@@ -16837,7 +16837,7 @@
       <c r="P302" t="inlineStr"/>
       <c r="Q302" t="inlineStr">
         <is>
-          <t>NOT SEEDED - compassmot compensation. Device-ID pinning table exists (ArduCopter/xplorer_compass_mot_pinning.h) but xplorer_compass_mot_boot_align() is CURRENTLY COMMENTED OUT in system.cpp (TEMP-COMPASS-EXPERIMENT) | should make false once we fix this on a lower level</t>
+          <t>NOT SEEDED in defaults.parm - value is written at boot by xplorer_compass_mot_boot_align() (system.cpp) from the device-ID-keyed table in ArduCopter/xplorer_compass_mot_pinning.h, which is the source of truth. Running CompassMot on a deployed unit will NOT persist across reboot; update the table and rebuild instead.</t>
         </is>
       </c>
       <c r="R302" t="inlineStr">
@@ -16898,7 +16898,7 @@
       <c r="P303" t="inlineStr"/>
       <c r="Q303" t="inlineStr">
         <is>
-          <t>NOT SEEDED - compassmot compensation. Device-ID pinning table exists (ArduCopter/xplorer_compass_mot_pinning.h) but xplorer_compass_mot_boot_align() is CURRENTLY COMMENTED OUT in system.cpp (TEMP-COMPASS-EXPERIMENT) | should make false once we fix this on a lower level</t>
+          <t>NOT SEEDED in defaults.parm - value is written at boot by xplorer_compass_mot_boot_align() (system.cpp) from the device-ID-keyed table in ArduCopter/xplorer_compass_mot_pinning.h, which is the source of truth. Running CompassMot on a deployed unit will NOT persist across reboot; update the table and rebuild instead.</t>
         </is>
       </c>
       <c r="R303" t="inlineStr">
@@ -17013,7 +17013,7 @@
       <c r="P305" t="inlineStr"/>
       <c r="Q305" t="inlineStr">
         <is>
-          <t>NOT SEEDED - compassmot compensation. Device-ID pinning table exists (ArduCopter/xplorer_compass_mot_pinning.h) but xplorer_compass_mot_boot_align() is CURRENTLY COMMENTED OUT in system.cpp (TEMP-COMPASS-EXPERIMENT) | should make false once we fix this on a lower level</t>
+          <t>NOT SEEDED in defaults.parm - value is written at boot by xplorer_compass_mot_boot_align() (system.cpp) from the device-ID-keyed table in ArduCopter/xplorer_compass_mot_pinning.h, which is the source of truth. Running CompassMot on a deployed unit will NOT persist across reboot; update the table and rebuild instead.</t>
         </is>
       </c>
       <c r="R305" t="inlineStr">
@@ -17074,7 +17074,7 @@
       <c r="P306" t="inlineStr"/>
       <c r="Q306" t="inlineStr">
         <is>
-          <t>NOT SEEDED - compassmot compensation. Device-ID pinning table exists (ArduCopter/xplorer_compass_mot_pinning.h) but xplorer_compass_mot_boot_align() is CURRENTLY COMMENTED OUT in system.cpp (TEMP-COMPASS-EXPERIMENT) | should make false once we fix this on a lower level</t>
+          <t>NOT SEEDED in defaults.parm - value is written at boot by xplorer_compass_mot_boot_align() (system.cpp) from the device-ID-keyed table in ArduCopter/xplorer_compass_mot_pinning.h, which is the source of truth. Running CompassMot on a deployed unit will NOT persist across reboot; update the table and rebuild instead.</t>
         </is>
       </c>
       <c r="R306" t="inlineStr">
@@ -17135,7 +17135,7 @@
       <c r="P307" t="inlineStr"/>
       <c r="Q307" t="inlineStr">
         <is>
-          <t>NOT SEEDED - compassmot compensation. Device-ID pinning table exists (ArduCopter/xplorer_compass_mot_pinning.h) but xplorer_compass_mot_boot_align() is CURRENTLY COMMENTED OUT in system.cpp (TEMP-COMPASS-EXPERIMENT) | should make false once we fix this on a lower level</t>
+          <t>NOT SEEDED in defaults.parm - value is written at boot by xplorer_compass_mot_boot_align() (system.cpp) from the device-ID-keyed table in ArduCopter/xplorer_compass_mot_pinning.h, which is the source of truth. Running CompassMot on a deployed unit will NOT persist across reboot; update the table and rebuild instead.</t>
         </is>
       </c>
       <c r="R307" t="inlineStr">
@@ -18238,7 +18238,7 @@
         </is>
       </c>
       <c r="C328" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D328" t="b">
         <v>0</v>
@@ -18271,7 +18271,7 @@
       <c r="P328" t="inlineStr"/>
       <c r="Q328" t="inlineStr">
         <is>
-          <t>defaults.parm: # TEMP-COMPASS-EXPERIMENT unlocked</t>
+          <t>defaults.parm: # TEMP-COMPASS-EXPERIMENT unlocked | 8 (Roll180) is the Ark Mag's mounting orientation, valid because slot 1 is pinned to it by COMPASS_PRIO1_ID. Orientation is slot-keyed, so this value is only correct as long as that pin holds.</t>
         </is>
       </c>
       <c r="R328" t="inlineStr">
@@ -18450,7 +18450,7 @@
         </is>
       </c>
       <c r="C332" t="n">
-        <v>96515</v>
+        <v>96259</v>
       </c>
       <c r="D332" t="b">
         <v>0</v>
@@ -18483,7 +18483,7 @@
       </c>
       <c r="Q332" t="inlineStr">
         <is>
-          <t>defaults.parm: # TEMP-COMPASS-EXPERIMENT unlocked</t>
+          <t>defaults.parm: # TEMP-COMPASS-EXPERIMENT unlocked | Hard-pinned to the Ark Mag (devid 96259 = DroneCAN node 120, sensor 0). Node ID is statically set on the peripheral and both CAN ports map to driver 1, so this devid is a design constant, not DNA-dependent.</t>
         </is>
       </c>
       <c r="R332" t="inlineStr">
@@ -18504,7 +18504,7 @@
         </is>
       </c>
       <c r="C333" t="n">
-        <v>162051</v>
+        <v>96515</v>
       </c>
       <c r="D333" t="b">
         <v>0</v>
@@ -18537,7 +18537,7 @@
       </c>
       <c r="Q333" t="inlineStr">
         <is>
-          <t>defaults.parm: # TEMP-COMPASS-EXPERIMENT unlocked</t>
+          <t>defaults.parm: # TEMP-COMPASS-EXPERIMENT unlocked | Hard-pinned to the Here4 primary (devid 96515 = DroneCAN node 121, sensor 0). Static node ID, same reasoning as COMPASS_PRIO1_ID.</t>
         </is>
       </c>
       <c r="R333" t="inlineStr">
@@ -18558,7 +18558,7 @@
         </is>
       </c>
       <c r="C334" t="n">
-        <v>1313809</v>
+        <v>0</v>
       </c>
       <c r="D334" t="b">
         <v>0</v>
@@ -18591,7 +18591,7 @@
       </c>
       <c r="Q334" t="inlineStr">
         <is>
-          <t>defaults.parm: # TEMP-COMPASS-EXPERIMENT unlocked</t>
+          <t>defaults.parm: # TEMP-COMPASS-EXPERIMENT unlocked | Deliberately seeded 0 (FLOATING). Slot 3 holds the Cube internal mag on airframes with an older single-compass Here4 (RM3100 only), and the Here4 second compass (devid 162051) on airframes with the newer dual-compass Here4, so no single value is correct for both. It self-pins per unit on first boot. Safe because USE3=0 and every device that can land there has a zero MOT entry in the pinning table.</t>
         </is>
       </c>
       <c r="R334" t="inlineStr">
@@ -69634,7 +69634,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-14 15:19 UTC</t>
+          <t>2026-09-02 17:34 UTC</t>
         </is>
       </c>
     </row>
@@ -69646,7 +69646,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>4864a04323</t>
+          <t>561e54fe3b</t>
         </is>
       </c>
     </row>
@@ -69670,7 +69670,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>xplorer-fw-v1.0.1-1-g4864a04323-dirty</t>
+          <t>xplorer-fw-v1.0.1-7-g561e54fe3b-dirty</t>
         </is>
       </c>
     </row>

</xml_diff>